<commit_message>
Excel file upload error handling and message feedback
</commit_message>
<xml_diff>
--- a/documents/SADV collections upload.xlsx
+++ b/documents/SADV collections upload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E4D753-C574-464A-80DA-BDF40B78BE80}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10BAE12-9B35-E549-A451-CCF36BEE59E5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="16000" xr2:uid="{B1A7F133-870B-BE4E-A664-D1E75F837A44}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="240">
   <si>
     <t>accountRef</t>
   </si>
@@ -1482,8 +1482,8 @@
       <c r="I5">
         <v>17250</v>
       </c>
-      <c r="J5" t="s">
-        <v>87</v>
+      <c r="J5">
+        <v>0</v>
       </c>
       <c r="K5" t="s">
         <v>27</v>
@@ -1962,8 +1962,8 @@
       <c r="I14">
         <v>0</v>
       </c>
-      <c r="J14" t="s">
-        <v>87</v>
+      <c r="J14">
+        <v>0</v>
       </c>
       <c r="K14" t="s">
         <v>27</v>
@@ -2018,8 +2018,8 @@
       <c r="I15">
         <v>0</v>
       </c>
-      <c r="J15" t="s">
-        <v>87</v>
+      <c r="J15">
+        <v>0</v>
       </c>
       <c r="K15" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Work on Collection.js to get the dates to show properly. Also some work on the import of dates in ExcelReader.js
</commit_message>
<xml_diff>
--- a/documents/SADV collections upload.xlsx
+++ b/documents/SADV collections upload.xlsx
@@ -8,13 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10BAE12-9B35-E549-A451-CCF36BEE59E5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC881B-6BCF-AA4C-88B6-58FDB91C6689}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="16000" xr2:uid="{B1A7F133-870B-BE4E-A664-D1E75F837A44}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AC$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet2!$A$1:$C$44</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -33,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="241">
   <si>
     <t>accountRef</t>
   </si>
@@ -287,9 +292,6 @@
     <t>30</t>
   </si>
   <si>
-    <t>O</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -665,9 +667,6 @@
     <t>Brittany Kruis</t>
   </si>
   <si>
-    <t>0878973950 / 0832758844</t>
-  </si>
-  <si>
     <t>Nazeer Khan</t>
   </si>
   <si>
@@ -701,9 +700,6 @@
     <t>JOSHUA VAN TONDER</t>
   </si>
   <si>
-    <t>0112830000/0827760859</t>
-  </si>
-  <si>
     <t>Charl Cockcroft</t>
   </si>
   <si>
@@ -753,13 +749,25 @@
   </si>
   <si>
     <t>RIAAN LUBBE</t>
+  </si>
+  <si>
+    <t># name</t>
+  </si>
+  <si>
+    <t>0878973950 / 0832758845</t>
+  </si>
+  <si>
+    <t>0112830000/0827760860</t>
+  </si>
+  <si>
+    <t>n/a</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -791,6 +799,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -800,7 +814,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -868,11 +882,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -895,6 +922,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,138 +1237,141 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264374CA-EBDB-1348-8948-C7AE36E6EA27}">
-  <dimension ref="A1:AB51"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:AD51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="63.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="3.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="14" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="41" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="63.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="41" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="23.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>31</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>33</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="12" t="str">
+        <f>VLOOKUP(A2,Sheet2!B2:B44,1,0)</f>
+        <v>EDG102</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
         <v>3500000</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
       <c r="H2">
         <v>0</v>
       </c>
@@ -1348,52 +1379,56 @@
         <v>0</v>
       </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
         <v>3500000</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
         <v>37457</v>
       </c>
-      <c r="V2" t="s">
-        <v>103</v>
-      </c>
       <c r="W2" t="s">
+        <v>102</v>
+      </c>
+      <c r="X2" t="s">
         <v>26</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>29</v>
       </c>
-      <c r="Y2" t="s">
-        <v>150</v>
-      </c>
       <c r="Z2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA2" t="s">
         <v>30</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>32</v>
       </c>
-      <c r="AB2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AC2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="12" t="e">
+        <f>VLOOKUP(A3,Sheet2!B3:B45,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
       <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>87175.63</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
       <c r="H3">
         <v>0</v>
       </c>
@@ -1401,39 +1436,43 @@
         <v>0</v>
       </c>
       <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
         <v>87175.63</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>27</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
+        <v>102</v>
+      </c>
+      <c r="X3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y3" t="s">
         <v>103</v>
       </c>
-      <c r="W3" t="s">
-        <v>34</v>
-      </c>
-      <c r="X3" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="12" t="e">
+        <f>VLOOKUP(A4,Sheet2!B4:B46,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
       <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
         <v>58919.59</v>
-      </c>
-      <c r="G4">
-        <v>2381.65</v>
       </c>
       <c r="H4">
         <v>2381.65</v>
@@ -1442,39 +1481,43 @@
         <v>2381.65</v>
       </c>
       <c r="J4">
+        <v>2381.65</v>
+      </c>
+      <c r="K4">
         <v>51774.64</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>27</v>
       </c>
-      <c r="V4" t="s">
-        <v>103</v>
-      </c>
       <c r="W4" t="s">
+        <v>102</v>
+      </c>
+      <c r="X4" t="s">
         <v>35</v>
       </c>
-      <c r="X4" t="s">
-        <v>105</v>
-      </c>
       <c r="Y4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="12" t="str">
+        <f>VLOOKUP(A5,Sheet2!B5:B47,1,0)</f>
+        <v>DWK101</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>51750</v>
-      </c>
-      <c r="G5">
-        <v>17250</v>
       </c>
       <c r="H5">
         <v>17250</v>
@@ -1483,102 +1526,110 @@
         <v>17250</v>
       </c>
       <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
+        <v>17250</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
         <v>27</v>
       </c>
-      <c r="V5" t="s">
-        <v>103</v>
-      </c>
       <c r="W5" t="s">
+        <v>102</v>
+      </c>
+      <c r="X5" t="s">
         <v>36</v>
       </c>
-      <c r="X5" t="s">
-        <v>106</v>
-      </c>
       <c r="Y5" t="s">
+        <v>105</v>
+      </c>
+      <c r="Z5" t="s">
         <v>28</v>
       </c>
-      <c r="Z5" t="s">
-        <v>151</v>
-      </c>
       <c r="AA5" t="s">
-        <v>189</v>
-      </c>
-      <c r="AB5">
+        <v>150</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC5">
         <v>114695876</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="12" t="str">
+        <f>VLOOKUP(A6,Sheet2!B6:B48,1,0)</f>
+        <v>SER103</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
       <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
         <v>47904.91</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>3187.34</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>6325.69</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>10628.3</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>27763.58</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>27</v>
       </c>
-      <c r="N6" s="3">
+      <c r="O6" s="3">
         <v>47228</v>
       </c>
-      <c r="V6" t="s">
-        <v>103</v>
-      </c>
       <c r="W6" t="s">
+        <v>102</v>
+      </c>
+      <c r="X6" t="s">
         <v>37</v>
       </c>
-      <c r="X6" t="s">
-        <v>107</v>
-      </c>
       <c r="Y6" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z6" t="s">
         <v>28</v>
       </c>
-      <c r="Z6" t="s">
-        <v>89</v>
-      </c>
       <c r="AA6" t="s">
-        <v>190</v>
-      </c>
-      <c r="AB6">
+        <v>88</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>189</v>
+      </c>
+      <c r="AC6">
         <v>115527000</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="12" t="str">
+        <f>VLOOKUP(A7,Sheet2!B7:B49,1,0)</f>
+        <v>REV101</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
       <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
         <v>40919.9</v>
       </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
       <c r="H7">
         <v>0</v>
       </c>
@@ -1586,52 +1637,56 @@
         <v>0</v>
       </c>
       <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>40919.9</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="3">
+      <c r="O7" s="3">
         <v>36968</v>
       </c>
-      <c r="V7" t="s">
-        <v>103</v>
-      </c>
       <c r="W7" t="s">
+        <v>102</v>
+      </c>
+      <c r="X7" t="s">
         <v>38</v>
       </c>
-      <c r="X7" t="s">
-        <v>108</v>
-      </c>
       <c r="Y7" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z7" t="s">
         <v>28</v>
       </c>
-      <c r="Z7" t="s">
-        <v>152</v>
-      </c>
       <c r="AA7" t="s">
-        <v>191</v>
-      </c>
-      <c r="AB7">
+        <v>151</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>190</v>
+      </c>
+      <c r="AC7">
         <v>786737791</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8">
+      <c r="B8" s="12" t="e">
+        <f>VLOOKUP(A8,Sheet2!B8:B50,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C8" s="2">
         <v>0</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>37986.800000000003</v>
       </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
       <c r="H8">
         <v>0</v>
       </c>
@@ -1639,52 +1694,56 @@
         <v>0</v>
       </c>
       <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
         <v>37986.800000000003</v>
       </c>
-      <c r="K8" t="s">
-        <v>88</v>
-      </c>
-      <c r="N8" s="3">
+      <c r="L8" t="s">
+        <v>87</v>
+      </c>
+      <c r="O8" s="3">
         <v>38278</v>
       </c>
-      <c r="V8" t="s">
-        <v>103</v>
-      </c>
       <c r="W8" t="s">
+        <v>102</v>
+      </c>
+      <c r="X8" t="s">
         <v>39</v>
       </c>
-      <c r="X8" t="s">
-        <v>109</v>
-      </c>
       <c r="Y8" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z8" t="s">
         <v>28</v>
       </c>
-      <c r="Z8" t="s">
-        <v>153</v>
-      </c>
       <c r="AA8" t="s">
-        <v>192</v>
-      </c>
-      <c r="AB8">
+        <v>152</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>191</v>
+      </c>
+      <c r="AC8">
         <v>823314531</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="12" t="str">
+        <f>VLOOKUP(A9,Sheet2!B9:B51,1,0)</f>
+        <v>ALJ101</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
       <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
         <v>34658.080000000002</v>
       </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
       <c r="H9">
         <v>0</v>
       </c>
@@ -1692,158 +1751,170 @@
         <v>0</v>
       </c>
       <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>34658.080000000002</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>27</v>
       </c>
-      <c r="V9" t="s">
-        <v>103</v>
-      </c>
       <c r="W9" t="s">
+        <v>102</v>
+      </c>
+      <c r="X9" t="s">
         <v>40</v>
       </c>
-      <c r="X9" t="s">
-        <v>110</v>
-      </c>
       <c r="Y9" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z9" t="s">
         <v>28</v>
       </c>
-      <c r="Z9" t="s">
-        <v>154</v>
-      </c>
       <c r="AA9" t="s">
-        <v>193</v>
-      </c>
-      <c r="AB9">
+        <v>153</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>192</v>
+      </c>
+      <c r="AC9">
         <v>790600367</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="12" t="str">
+        <f>VLOOKUP(A10,Sheet2!B10:B52,1,0)</f>
+        <v>BEBR01</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
       <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
         <v>535444.18000000005</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>147152.29</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>263114.37</v>
       </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
       <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
         <v>125177.52</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="3">
+      <c r="O10" s="3">
         <v>38918</v>
       </c>
-      <c r="R10" t="s">
-        <v>90</v>
-      </c>
-      <c r="V10" t="s">
-        <v>103</v>
+      <c r="S10" t="s">
+        <v>89</v>
       </c>
       <c r="W10" t="s">
+        <v>102</v>
+      </c>
+      <c r="X10" t="s">
         <v>41</v>
       </c>
-      <c r="X10" t="s">
-        <v>111</v>
-      </c>
       <c r="Y10" t="s">
-        <v>150</v>
+        <v>110</v>
       </c>
       <c r="Z10" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="AA10" t="s">
-        <v>194</v>
-      </c>
-      <c r="AB10">
+        <v>154</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>193</v>
+      </c>
+      <c r="AC10">
         <v>663023759</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="12" t="str">
+        <f>VLOOKUP(A11,Sheet2!B11:B53,1,0)</f>
+        <v>AFRI10</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
       <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
         <v>316090.96999999997</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>100580.42</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>166871.19</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
       <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
         <v>48639.360000000001</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="3">
+      <c r="O11" s="3">
         <v>11068</v>
       </c>
-      <c r="R11" t="s">
-        <v>90</v>
-      </c>
-      <c r="V11" t="s">
-        <v>103</v>
+      <c r="S11" t="s">
+        <v>89</v>
       </c>
       <c r="W11" t="s">
+        <v>102</v>
+      </c>
+      <c r="X11" t="s">
         <v>42</v>
       </c>
-      <c r="X11" t="s">
-        <v>112</v>
-      </c>
       <c r="Y11" t="s">
-        <v>150</v>
+        <v>111</v>
       </c>
       <c r="Z11" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="AA11" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="12" t="str">
+        <f>VLOOKUP(A12,Sheet2!B12:B54,1,0)</f>
+        <v>NEP101</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
       <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
         <v>193540.4</v>
       </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
       <c r="H12">
         <v>0</v>
       </c>
@@ -1851,279 +1922,299 @@
         <v>0</v>
       </c>
       <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
         <v>193540.4</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>27</v>
       </c>
-      <c r="N12" s="3">
+      <c r="O12" s="3">
         <v>11037</v>
       </c>
-      <c r="R12" t="s">
-        <v>90</v>
-      </c>
-      <c r="V12" t="s">
-        <v>103</v>
+      <c r="S12" t="s">
+        <v>89</v>
       </c>
       <c r="W12" t="s">
+        <v>102</v>
+      </c>
+      <c r="X12" t="s">
         <v>43</v>
       </c>
-      <c r="X12" t="s">
-        <v>113</v>
-      </c>
       <c r="Y12" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="Z12" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="AA12" t="s">
-        <v>196</v>
-      </c>
-      <c r="AB12">
+        <v>156</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>195</v>
+      </c>
+      <c r="AC12">
         <v>119797038</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="12" t="e">
+        <f>VLOOKUP(A13,Sheet2!B13:B55,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
       <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
         <v>160278.18</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>53618.83</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>86121.86</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
       <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
         <v>20537.490000000002</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>27</v>
       </c>
-      <c r="N13" s="3">
+      <c r="O13" s="3">
         <v>38127</v>
       </c>
-      <c r="R13" t="s">
-        <v>90</v>
-      </c>
-      <c r="V13" t="s">
-        <v>103</v>
+      <c r="S13" t="s">
+        <v>89</v>
       </c>
       <c r="W13" t="s">
+        <v>102</v>
+      </c>
+      <c r="X13" t="s">
         <v>44</v>
       </c>
-      <c r="X13" t="s">
-        <v>114</v>
-      </c>
       <c r="Y13" t="s">
-        <v>150</v>
+        <v>113</v>
       </c>
       <c r="Z13" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="AA13" t="s">
-        <v>197</v>
-      </c>
-      <c r="AB13">
+        <v>157</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>196</v>
+      </c>
+      <c r="AC13">
         <v>214649682</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="12" t="e">
+        <f>VLOOKUP(A14,Sheet2!B14:B56,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
       <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
         <v>151749.93</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>52277.25</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>99472.68</v>
       </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
       <c r="J14">
         <v>0</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14" t="s">
         <v>27</v>
       </c>
-      <c r="N14" s="3">
+      <c r="O14" s="3">
         <v>42906</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
+        <v>89</v>
+      </c>
+      <c r="W14" t="s">
+        <v>102</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA14" t="s">
         <v>90</v>
       </c>
-      <c r="V14" t="s">
-        <v>103</v>
-      </c>
-      <c r="W14" t="s">
-        <v>45</v>
-      </c>
-      <c r="X14" t="s">
-        <v>115</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>150</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>198</v>
-      </c>
-      <c r="AB14">
+      <c r="AB14" t="s">
+        <v>197</v>
+      </c>
+      <c r="AC14">
         <v>848373798</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="12" t="e">
+        <f>VLOOKUP(A15,Sheet2!B15:B57,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
       <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
         <v>131059.9</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>50821.87</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>80238.03</v>
       </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
       <c r="J15">
         <v>0</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="3">
+      <c r="O15" s="3">
         <v>11098</v>
       </c>
-      <c r="R15" t="s">
-        <v>90</v>
-      </c>
-      <c r="V15" t="s">
-        <v>103</v>
+      <c r="S15" t="s">
+        <v>89</v>
       </c>
       <c r="W15" t="s">
+        <v>102</v>
+      </c>
+      <c r="X15" t="s">
         <v>46</v>
       </c>
-      <c r="X15" t="s">
-        <v>116</v>
-      </c>
       <c r="Y15" t="s">
-        <v>150</v>
+        <v>115</v>
       </c>
       <c r="Z15" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="AA15" t="s">
-        <v>199</v>
-      </c>
-      <c r="AB15">
+        <v>158</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>198</v>
+      </c>
+      <c r="AC15">
         <v>214649682</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="12" t="e">
+        <f>VLOOKUP(A16,Sheet2!B16:B58,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
       <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
         <v>128836.85</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>724.5</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>1449</v>
       </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
       <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
         <v>126663.35</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>27</v>
       </c>
-      <c r="N16" s="3">
+      <c r="O16" s="3">
         <v>40683</v>
       </c>
-      <c r="R16" t="s">
-        <v>90</v>
-      </c>
-      <c r="V16" t="s">
-        <v>103</v>
+      <c r="S16" t="s">
+        <v>89</v>
       </c>
       <c r="W16" t="s">
+        <v>102</v>
+      </c>
+      <c r="X16" t="s">
         <v>47</v>
       </c>
-      <c r="X16" t="s">
-        <v>117</v>
-      </c>
       <c r="Y16" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="Z16" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="AA16" t="s">
-        <v>200</v>
-      </c>
-      <c r="AB16">
+        <v>159</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>199</v>
+      </c>
+      <c r="AC16">
         <v>100350005</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="12" t="str">
+        <f>VLOOKUP(A17,Sheet2!B17:B59,1,0)</f>
+        <v>SKYF01</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
       <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>127304.16</v>
       </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
       <c r="H17">
         <v>0</v>
       </c>
@@ -2131,167 +2222,179 @@
         <v>0</v>
       </c>
       <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
         <v>127304.16</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>27</v>
       </c>
-      <c r="N17" s="3">
+      <c r="O17" s="3">
         <v>37731</v>
       </c>
-      <c r="R17" t="s">
-        <v>90</v>
-      </c>
-      <c r="V17" t="s">
-        <v>103</v>
+      <c r="S17" t="s">
+        <v>89</v>
       </c>
       <c r="W17" t="s">
+        <v>102</v>
+      </c>
+      <c r="X17" t="s">
         <v>48</v>
       </c>
-      <c r="X17" t="s">
-        <v>118</v>
-      </c>
       <c r="Y17" t="s">
-        <v>150</v>
+        <v>117</v>
       </c>
       <c r="Z17" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="AA17" t="s">
-        <v>201</v>
-      </c>
-      <c r="AB17">
+        <v>160</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC17">
         <v>784299841</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="12" t="str">
+        <f>VLOOKUP(A18,Sheet2!B18:B60,1,0)</f>
+        <v>MWEB01</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
       <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
         <v>116868.58</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>72858.080000000002</v>
       </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
         <v>44010.5</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>27</v>
       </c>
-      <c r="N18" s="3">
+      <c r="O18" s="3">
         <v>11129</v>
       </c>
-      <c r="R18" t="s">
-        <v>90</v>
-      </c>
-      <c r="V18" t="s">
-        <v>103</v>
+      <c r="S18" t="s">
+        <v>89</v>
       </c>
       <c r="W18" t="s">
+        <v>102</v>
+      </c>
+      <c r="X18" t="s">
         <v>49</v>
       </c>
-      <c r="X18" t="s">
-        <v>119</v>
-      </c>
       <c r="Y18" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="Z18" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="AA18" t="s">
-        <v>202</v>
-      </c>
-      <c r="AB18">
+        <v>161</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>201</v>
+      </c>
+      <c r="AC18">
         <v>215968443</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="12" t="str">
+        <f>VLOOKUP(A19,Sheet2!B19:B61,1,0)</f>
+        <v>HC0101</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
       <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
         <v>106379.92</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>33281.870000000003</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>61765.75</v>
       </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
       <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
         <v>11332.3</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>27</v>
       </c>
-      <c r="N19" s="3">
+      <c r="O19" s="3">
         <v>43636</v>
       </c>
-      <c r="R19" t="s">
-        <v>90</v>
-      </c>
-      <c r="V19" t="s">
-        <v>103</v>
+      <c r="S19" t="s">
+        <v>89</v>
       </c>
       <c r="W19" t="s">
+        <v>102</v>
+      </c>
+      <c r="X19" t="s">
         <v>50</v>
       </c>
-      <c r="X19" t="s">
-        <v>120</v>
-      </c>
       <c r="Y19" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="Z19" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="AA19" t="s">
-        <v>203</v>
-      </c>
-      <c r="AB19">
+        <v>162</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>202</v>
+      </c>
+      <c r="AC19">
         <v>215968443</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="12" t="str">
+        <f>VLOOKUP(A20,Sheet2!B20:B62,1,0)</f>
+        <v>ACCG01</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
       <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
         <v>101296.03</v>
       </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
       <c r="H20">
         <v>0</v>
       </c>
@@ -2299,55 +2402,59 @@
         <v>0</v>
       </c>
       <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
         <v>101296.03</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>27</v>
       </c>
-      <c r="N20" s="3">
+      <c r="O20" s="3">
         <v>40683</v>
       </c>
-      <c r="R20" t="s">
-        <v>90</v>
-      </c>
-      <c r="V20" t="s">
-        <v>103</v>
+      <c r="S20" t="s">
+        <v>89</v>
       </c>
       <c r="W20" t="s">
+        <v>102</v>
+      </c>
+      <c r="X20" t="s">
         <v>51</v>
       </c>
-      <c r="X20" t="s">
-        <v>121</v>
-      </c>
       <c r="Y20" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="Z20" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="AA20" t="s">
-        <v>204</v>
-      </c>
-      <c r="AB20">
+        <v>163</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>203</v>
+      </c>
+      <c r="AC20">
         <v>853003000</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="12" t="str">
+        <f>VLOOKUP(A21,Sheet2!B21:B63,1,0)</f>
+        <v>LEGE01</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
       <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
         <v>90761.76</v>
       </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
       <c r="H21">
         <v>0</v>
       </c>
@@ -2355,384 +2462,415 @@
         <v>0</v>
       </c>
       <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
         <v>90761.76</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>27</v>
       </c>
-      <c r="N21" s="3">
+      <c r="O21" s="3">
         <v>37672</v>
       </c>
-      <c r="R21" t="s">
-        <v>90</v>
-      </c>
-      <c r="V21" t="s">
-        <v>103</v>
+      <c r="S21" t="s">
+        <v>89</v>
       </c>
       <c r="W21" t="s">
+        <v>102</v>
+      </c>
+      <c r="X21" t="s">
         <v>52</v>
       </c>
-      <c r="X21" t="s">
-        <v>122</v>
-      </c>
       <c r="Y21" t="s">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="Z21" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="AA21" t="s">
-        <v>205</v>
-      </c>
-      <c r="AB21">
+        <v>164</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>204</v>
+      </c>
+      <c r="AC21">
         <v>611064892</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="12" t="str">
+        <f>VLOOKUP(A22,Sheet2!B22:B64,1,0)</f>
+        <v>RD0101</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
       <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
         <v>65339.96</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>4255</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>8510</v>
       </c>
-      <c r="I22">
-        <v>0</v>
-      </c>
       <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
         <v>52574.96</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>27</v>
       </c>
-      <c r="N22" s="3">
+      <c r="O22" s="3">
         <v>38857</v>
       </c>
-      <c r="R22" t="s">
-        <v>90</v>
-      </c>
-      <c r="V22" t="s">
-        <v>103</v>
+      <c r="S22" t="s">
+        <v>89</v>
       </c>
       <c r="W22" t="s">
+        <v>102</v>
+      </c>
+      <c r="X22" t="s">
         <v>53</v>
       </c>
-      <c r="X22" t="s">
-        <v>123</v>
-      </c>
       <c r="Y22" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="Z22" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="AA22" t="s">
-        <v>206</v>
-      </c>
-      <c r="AB22">
+        <v>165</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>205</v>
+      </c>
+      <c r="AC22">
         <v>100150150</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="12" t="e">
+        <f>VLOOKUP(A23,Sheet2!B23:B65,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
       <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
         <v>56661.17</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>21397</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>35264.15</v>
       </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
       <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
         <v>0.02</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="3">
+      <c r="O23" s="3">
         <v>45402</v>
       </c>
-      <c r="R23" t="s">
-        <v>90</v>
-      </c>
-      <c r="V23" t="s">
-        <v>103</v>
+      <c r="S23" t="s">
+        <v>89</v>
       </c>
       <c r="W23" t="s">
+        <v>102</v>
+      </c>
+      <c r="X23" t="s">
         <v>54</v>
       </c>
-      <c r="X23" t="s">
-        <v>124</v>
-      </c>
       <c r="Y23" t="s">
-        <v>150</v>
+        <v>123</v>
       </c>
       <c r="Z23" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="AA23" t="s">
-        <v>207</v>
-      </c>
-      <c r="AB23">
+        <v>166</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>206</v>
+      </c>
+      <c r="AC23">
         <v>126793423</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="12" t="str">
+        <f>VLOOKUP(A24,Sheet2!B24:B66,1,0)</f>
+        <v>HXS101</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
       <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>37173.75</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>7820</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>15640</v>
       </c>
-      <c r="I24">
-        <v>0</v>
-      </c>
       <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>13713.75</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="3">
+      <c r="O24" s="3">
         <v>40622</v>
       </c>
-      <c r="R24" t="s">
-        <v>90</v>
-      </c>
-      <c r="V24" t="s">
-        <v>103</v>
+      <c r="S24" t="s">
+        <v>89</v>
       </c>
       <c r="W24" t="s">
+        <v>102</v>
+      </c>
+      <c r="X24" t="s">
         <v>55</v>
       </c>
-      <c r="X24" t="s">
-        <v>125</v>
-      </c>
       <c r="Y24" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
       <c r="Z24" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="AA24" t="s">
-        <v>208</v>
-      </c>
-      <c r="AB24">
+        <v>167</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>207</v>
+      </c>
+      <c r="AC24">
         <v>791494245</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="12" t="e">
+        <f>VLOOKUP(A25,Sheet2!B25:B67,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
       <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>2086473.5</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>140609.5</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>152756.25</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>146566.24</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>1646541.51</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>27</v>
       </c>
-      <c r="R25" t="s">
-        <v>91</v>
-      </c>
-      <c r="V25" t="s">
-        <v>103</v>
+      <c r="S25" t="s">
+        <v>90</v>
       </c>
       <c r="W25" t="s">
+        <v>102</v>
+      </c>
+      <c r="X25" t="s">
         <v>56</v>
       </c>
-      <c r="X25" t="s">
-        <v>126</v>
-      </c>
       <c r="Y25" t="s">
-        <v>169</v>
+        <v>125</v>
       </c>
       <c r="Z25" t="s">
-        <v>91</v>
+        <v>168</v>
       </c>
       <c r="AA25" t="s">
-        <v>209</v>
+        <v>90</v>
       </c>
       <c r="AB25" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+      <c r="AC25">
+        <v>878973950</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="12" t="e">
+        <f>VLOOKUP(A26,Sheet2!B26:B68,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
       <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
         <v>511727.12</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>203937.7</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>214970.03</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>92819.39</v>
       </c>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26" t="s">
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26" t="s">
         <v>27</v>
       </c>
-      <c r="R26" t="s">
-        <v>89</v>
-      </c>
-      <c r="V26" t="s">
-        <v>103</v>
+      <c r="S26" t="s">
+        <v>88</v>
       </c>
       <c r="W26" t="s">
+        <v>102</v>
+      </c>
+      <c r="X26" t="s">
         <v>57</v>
       </c>
-      <c r="X26" t="s">
-        <v>127</v>
-      </c>
       <c r="Y26" t="s">
+        <v>126</v>
+      </c>
+      <c r="Z26" t="s">
         <v>28</v>
       </c>
-      <c r="Z26" t="s">
-        <v>91</v>
-      </c>
       <c r="AA26" t="s">
-        <v>211</v>
-      </c>
-      <c r="AB26">
+        <v>90</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>209</v>
+      </c>
+      <c r="AC26">
         <v>124431000</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
+      <c r="B27" s="12" t="e">
+        <f>VLOOKUP(A27,Sheet2!B27:B69,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
         <v>257112.85</v>
       </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
       <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
         <v>48767.08</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>50823.94</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>157521.82999999999</v>
       </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
         <v>27</v>
       </c>
-      <c r="N27" s="3">
+      <c r="O27" s="3">
         <v>47289</v>
       </c>
-      <c r="R27" t="s">
-        <v>89</v>
-      </c>
-      <c r="V27" t="s">
-        <v>103</v>
+      <c r="S27" t="s">
+        <v>88</v>
       </c>
       <c r="W27" t="s">
+        <v>102</v>
+      </c>
+      <c r="X27" t="s">
         <v>58</v>
       </c>
-      <c r="X27" t="s">
-        <v>128</v>
-      </c>
       <c r="Y27" t="s">
+        <v>127</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>168</v>
+      </c>
+      <c r="AA27" t="s">
         <v>169</v>
       </c>
-      <c r="Z27" t="s">
-        <v>170</v>
-      </c>
-      <c r="AA27" t="s">
-        <v>212</v>
-      </c>
-      <c r="AB27">
+      <c r="AB27" t="s">
+        <v>210</v>
+      </c>
+      <c r="AC27">
         <v>101610660</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="12" t="str">
+        <f>VLOOKUP(A28,Sheet2!B28:B70,1,0)</f>
+        <v>GAL101</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
       <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
         <v>103781.75</v>
-      </c>
-      <c r="G28">
-        <v>20756.349999999999</v>
       </c>
       <c r="H28">
         <v>20756.349999999999</v>
@@ -2741,110 +2879,118 @@
         <v>20756.349999999999</v>
       </c>
       <c r="J28">
+        <v>20756.349999999999</v>
+      </c>
+      <c r="K28">
         <v>41512.699999999997</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>27</v>
       </c>
-      <c r="N28" s="3">
+      <c r="O28" s="3">
         <v>39133</v>
       </c>
-      <c r="R28" t="s">
-        <v>92</v>
-      </c>
-      <c r="V28" t="s">
-        <v>103</v>
+      <c r="S28" t="s">
+        <v>91</v>
       </c>
       <c r="W28" t="s">
+        <v>102</v>
+      </c>
+      <c r="X28" t="s">
         <v>59</v>
       </c>
-      <c r="X28" t="s">
-        <v>129</v>
-      </c>
       <c r="Y28" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z28" t="s">
         <v>28</v>
       </c>
-      <c r="Z28" t="s">
-        <v>171</v>
-      </c>
       <c r="AA28" t="s">
-        <v>213</v>
-      </c>
-      <c r="AB28">
+        <v>170</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>211</v>
+      </c>
+      <c r="AC28">
         <v>828517094</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="12" t="e">
+        <f>VLOOKUP(A29,Sheet2!B29:B71,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
       <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
         <v>49552.35</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>49552.35</v>
       </c>
-      <c r="H29">
-        <v>0</v>
-      </c>
       <c r="I29">
         <v>0</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29" t="s">
         <v>27</v>
       </c>
-      <c r="N29" s="3">
+      <c r="O29" s="3">
         <v>45828</v>
       </c>
-      <c r="R29" t="s">
-        <v>93</v>
-      </c>
-      <c r="V29" t="s">
-        <v>103</v>
+      <c r="S29" t="s">
+        <v>92</v>
       </c>
       <c r="W29" t="s">
+        <v>102</v>
+      </c>
+      <c r="X29" t="s">
         <v>60</v>
       </c>
-      <c r="X29" t="s">
-        <v>130</v>
-      </c>
       <c r="Y29" t="s">
+        <v>129</v>
+      </c>
+      <c r="Z29" t="s">
         <v>28</v>
       </c>
-      <c r="Z29" t="s">
-        <v>172</v>
-      </c>
       <c r="AA29" t="s">
-        <v>214</v>
-      </c>
-      <c r="AB29">
+        <v>171</v>
+      </c>
+      <c r="AB29" t="s">
+        <v>212</v>
+      </c>
+      <c r="AC29">
         <v>115193000</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="12" t="e">
+        <f>VLOOKUP(A30,Sheet2!B30:B72,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
       <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
         <v>46133.4</v>
-      </c>
-      <c r="G30">
-        <v>15377.8</v>
       </c>
       <c r="H30">
         <v>15377.8</v>
@@ -2853,55 +2999,59 @@
         <v>15377.8</v>
       </c>
       <c r="J30">
-        <v>0</v>
-      </c>
-      <c r="K30" t="s">
+        <v>15377.8</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30" t="s">
         <v>27</v>
       </c>
-      <c r="N30" s="3">
+      <c r="O30" s="3">
         <v>43240</v>
       </c>
-      <c r="R30" t="s">
-        <v>89</v>
-      </c>
-      <c r="V30" t="s">
-        <v>103</v>
+      <c r="S30" t="s">
+        <v>88</v>
       </c>
       <c r="W30" t="s">
+        <v>102</v>
+      </c>
+      <c r="X30" t="s">
         <v>61</v>
       </c>
-      <c r="X30" t="s">
-        <v>131</v>
-      </c>
       <c r="Y30" t="s">
+        <v>130</v>
+      </c>
+      <c r="Z30" t="s">
         <v>28</v>
       </c>
-      <c r="Z30" t="s">
-        <v>173</v>
-      </c>
       <c r="AA30" t="s">
-        <v>215</v>
-      </c>
-      <c r="AB30">
+        <v>172</v>
+      </c>
+      <c r="AB30" t="s">
+        <v>213</v>
+      </c>
+      <c r="AC30">
         <v>115851000</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31">
+      <c r="B31" s="12" t="e">
+        <f>VLOOKUP(A31,Sheet2!B31:B73,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C31" s="2">
         <v>0</v>
       </c>
       <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
         <v>39281.919999999998</v>
       </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
       <c r="H31">
         <v>0</v>
       </c>
@@ -2909,55 +3059,59 @@
         <v>0</v>
       </c>
       <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
         <v>39281.919999999998</v>
       </c>
-      <c r="K31" t="s">
-        <v>88</v>
-      </c>
-      <c r="N31" s="3">
+      <c r="L31" t="s">
+        <v>87</v>
+      </c>
+      <c r="O31" s="3">
         <v>37641</v>
       </c>
-      <c r="R31" t="s">
-        <v>94</v>
-      </c>
-      <c r="V31" t="s">
-        <v>103</v>
+      <c r="S31" t="s">
+        <v>93</v>
       </c>
       <c r="W31" t="s">
+        <v>102</v>
+      </c>
+      <c r="X31" t="s">
         <v>62</v>
       </c>
-      <c r="X31" t="s">
-        <v>132</v>
-      </c>
       <c r="Y31" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>173</v>
+      </c>
+      <c r="AA31" t="s">
         <v>174</v>
       </c>
-      <c r="Z31" t="s">
-        <v>175</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>132</v>
-      </c>
-      <c r="AB31">
+      <c r="AB31" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC31">
         <v>604821967</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="12" t="e">
+        <f>VLOOKUP(A32,Sheet2!B32:B74,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
       <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
         <v>32478.880000000001</v>
       </c>
-      <c r="G32">
-        <v>0</v>
-      </c>
       <c r="H32">
         <v>0</v>
       </c>
@@ -2965,52 +3119,59 @@
         <v>0</v>
       </c>
       <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
         <v>32478.880000000001</v>
       </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
         <v>27</v>
       </c>
-      <c r="N32" s="3">
+      <c r="O32" s="3">
         <v>37183</v>
       </c>
-      <c r="R32" t="s">
-        <v>95</v>
-      </c>
-      <c r="V32" t="s">
-        <v>103</v>
+      <c r="S32" t="s">
+        <v>94</v>
       </c>
       <c r="W32" t="s">
+        <v>102</v>
+      </c>
+      <c r="X32" t="s">
         <v>63</v>
       </c>
       <c r="Y32" t="s">
+        <v>240</v>
+      </c>
+      <c r="Z32" t="s">
         <v>28</v>
       </c>
-      <c r="Z32" t="s">
-        <v>91</v>
-      </c>
       <c r="AA32" t="s">
-        <v>216</v>
-      </c>
-      <c r="AB32">
+        <v>90</v>
+      </c>
+      <c r="AB32" t="s">
+        <v>214</v>
+      </c>
+      <c r="AC32">
         <v>114474360</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="12" t="e">
+        <f>VLOOKUP(A33,Sheet2!B33:B75,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
       <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
         <v>876306.58</v>
       </c>
-      <c r="G33">
-        <v>0</v>
-      </c>
       <c r="H33">
         <v>0</v>
       </c>
@@ -3018,55 +3179,59 @@
         <v>0</v>
       </c>
       <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
         <v>876306.58</v>
       </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
         <v>27</v>
       </c>
-      <c r="N33" s="3">
+      <c r="O33" s="3">
         <v>11129</v>
       </c>
-      <c r="R33" t="s">
-        <v>95</v>
-      </c>
-      <c r="V33" t="s">
-        <v>103</v>
+      <c r="S33" t="s">
+        <v>94</v>
       </c>
       <c r="W33" t="s">
+        <v>102</v>
+      </c>
+      <c r="X33" t="s">
         <v>64</v>
       </c>
-      <c r="X33" t="s">
-        <v>133</v>
-      </c>
       <c r="Y33" t="s">
+        <v>132</v>
+      </c>
+      <c r="Z33" t="s">
         <v>28</v>
       </c>
-      <c r="Z33" t="s">
-        <v>89</v>
-      </c>
       <c r="AA33" t="s">
-        <v>217</v>
+        <v>88</v>
       </c>
       <c r="AB33" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="34" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C34">
-        <v>0</v>
+      <c r="B34" s="12" t="str">
+        <f>VLOOKUP(A34,Sheet2!B34:B76,1,0)</f>
+        <v>AKH101</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
         <v>423300.2</v>
       </c>
-      <c r="G34">
-        <v>0</v>
-      </c>
       <c r="H34">
         <v>0</v>
       </c>
@@ -3074,166 +3239,181 @@
         <v>0</v>
       </c>
       <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
         <v>423300.2</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>27</v>
       </c>
-      <c r="N34" s="3">
+      <c r="O34" s="3">
         <v>38980</v>
       </c>
-      <c r="R34" t="s">
-        <v>96</v>
-      </c>
-      <c r="V34" t="s">
-        <v>103</v>
+      <c r="S34" t="s">
+        <v>95</v>
       </c>
       <c r="W34" t="s">
+        <v>102</v>
+      </c>
+      <c r="X34" t="s">
         <v>65</v>
       </c>
-      <c r="X34" t="s">
-        <v>134</v>
-      </c>
       <c r="Y34" t="s">
+        <v>133</v>
+      </c>
+      <c r="Z34" t="s">
         <v>28</v>
       </c>
-      <c r="Z34" t="s">
-        <v>176</v>
-      </c>
       <c r="AA34" t="s">
-        <v>219</v>
+        <v>175</v>
       </c>
       <c r="AB34" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="35" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="35" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="12" t="e">
+        <f>VLOOKUP(A35,Sheet2!B35:B77,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
       <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
         <v>229122.72</v>
       </c>
-      <c r="G35">
+      <c r="H35">
         <v>10.220000000000001</v>
       </c>
-      <c r="H35">
-        <v>0</v>
-      </c>
       <c r="I35">
         <v>0</v>
       </c>
       <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
         <v>229112.5</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="3">
+      <c r="O35" s="3">
         <v>11129</v>
       </c>
-      <c r="R35" t="s">
-        <v>95</v>
-      </c>
-      <c r="V35" t="s">
-        <v>103</v>
+      <c r="S35" t="s">
+        <v>94</v>
       </c>
       <c r="W35" t="s">
+        <v>102</v>
+      </c>
+      <c r="X35" t="s">
         <v>66</v>
       </c>
-      <c r="X35" t="s">
-        <v>135</v>
-      </c>
       <c r="Y35" t="s">
+        <v>134</v>
+      </c>
+      <c r="Z35" t="s">
         <v>28</v>
       </c>
-      <c r="Z35" t="s">
-        <v>177</v>
-      </c>
       <c r="AA35" t="s">
-        <v>221</v>
+        <v>176</v>
       </c>
       <c r="AB35" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="36" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+      <c r="AC35">
+        <v>112830000</v>
+      </c>
+      <c r="AD35" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="36" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
+      <c r="B36" s="12" t="e">
+        <f>VLOOKUP(A36,Sheet2!B36:B78,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
         <v>80497.7</v>
-      </c>
-      <c r="G36">
-        <v>40248.85</v>
       </c>
       <c r="H36">
         <v>40248.85</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>40248.85</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
-      <c r="K36" t="s">
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="L36" t="s">
         <v>27</v>
       </c>
-      <c r="N36" s="3">
+      <c r="O36" s="3">
         <v>40349</v>
       </c>
-      <c r="R36" t="s">
-        <v>97</v>
-      </c>
-      <c r="V36" t="s">
-        <v>103</v>
+      <c r="S36" t="s">
+        <v>96</v>
       </c>
       <c r="W36" t="s">
+        <v>102</v>
+      </c>
+      <c r="X36" t="s">
         <v>67</v>
       </c>
-      <c r="X36" t="s">
-        <v>136</v>
-      </c>
       <c r="Y36" t="s">
+        <v>135</v>
+      </c>
+      <c r="Z36" t="s">
         <v>28</v>
       </c>
-      <c r="Z36" t="s">
-        <v>178</v>
-      </c>
       <c r="AA36" t="s">
-        <v>223</v>
-      </c>
-      <c r="AB36">
+        <v>177</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>220</v>
+      </c>
+      <c r="AC36">
         <v>117450100</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="12" t="e">
+        <f>VLOOKUP(A37,Sheet2!B37:B79,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
       <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
         <v>68563</v>
-      </c>
-      <c r="G37">
-        <v>2116</v>
       </c>
       <c r="H37">
         <v>2116</v>
@@ -3242,160 +3422,172 @@
         <v>2116</v>
       </c>
       <c r="J37">
+        <v>2116</v>
+      </c>
+      <c r="K37">
         <v>62215</v>
       </c>
-      <c r="K37" t="s">
+      <c r="L37" t="s">
         <v>27</v>
       </c>
-      <c r="R37" t="s">
-        <v>96</v>
-      </c>
-      <c r="V37" t="s">
-        <v>103</v>
+      <c r="S37" t="s">
+        <v>95</v>
       </c>
       <c r="W37" t="s">
+        <v>102</v>
+      </c>
+      <c r="X37" t="s">
         <v>68</v>
       </c>
-      <c r="X37" t="s">
-        <v>137</v>
-      </c>
       <c r="Y37" t="s">
+        <v>136</v>
+      </c>
+      <c r="Z37" t="s">
         <v>28</v>
       </c>
-      <c r="Z37" t="s">
-        <v>89</v>
-      </c>
       <c r="AA37" t="s">
-        <v>224</v>
-      </c>
-      <c r="AB37">
+        <v>88</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>221</v>
+      </c>
+      <c r="AC37">
         <v>119123000</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="12" t="e">
+        <f>VLOOKUP(A38,Sheet2!B38:B80,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
       <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
         <v>55492</v>
       </c>
-      <c r="G38">
+      <c r="H38">
         <v>19169</v>
       </c>
-      <c r="H38">
+      <c r="I38">
         <v>36323</v>
       </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
       <c r="J38">
         <v>0</v>
       </c>
-      <c r="K38" t="s">
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38" t="s">
         <v>27</v>
       </c>
-      <c r="R38" t="s">
-        <v>98</v>
-      </c>
-      <c r="V38" t="s">
-        <v>103</v>
+      <c r="S38" t="s">
+        <v>97</v>
       </c>
       <c r="W38" t="s">
+        <v>102</v>
+      </c>
+      <c r="X38" t="s">
         <v>69</v>
       </c>
-      <c r="X38" t="s">
-        <v>138</v>
-      </c>
       <c r="Y38" t="s">
+        <v>137</v>
+      </c>
+      <c r="Z38" t="s">
         <v>28</v>
       </c>
-      <c r="Z38" t="s">
-        <v>179</v>
-      </c>
       <c r="AA38" t="s">
-        <v>225</v>
-      </c>
-      <c r="AB38">
+        <v>178</v>
+      </c>
+      <c r="AB38" t="s">
+        <v>222</v>
+      </c>
+      <c r="AC38">
         <v>100107301</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="12" t="e">
+        <f>VLOOKUP(A39,Sheet2!B39:B81,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
       <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
         <v>48467.9</v>
       </c>
-      <c r="G39">
+      <c r="H39">
         <v>6438.85</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>12187.7</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>6438.85</v>
       </c>
-      <c r="J39">
+      <c r="K39">
         <v>23402.5</v>
       </c>
-      <c r="K39" t="s">
+      <c r="L39" t="s">
         <v>27</v>
       </c>
-      <c r="N39" s="3">
+      <c r="O39" s="3">
         <v>46558</v>
       </c>
-      <c r="R39" t="s">
-        <v>95</v>
-      </c>
-      <c r="V39" t="s">
-        <v>103</v>
+      <c r="S39" t="s">
+        <v>94</v>
       </c>
       <c r="W39" t="s">
+        <v>102</v>
+      </c>
+      <c r="X39" t="s">
         <v>70</v>
       </c>
-      <c r="X39" t="s">
-        <v>139</v>
-      </c>
       <c r="Y39" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z39" t="s">
         <v>28</v>
       </c>
-      <c r="Z39" t="s">
-        <v>180</v>
-      </c>
       <c r="AA39" t="s">
-        <v>226</v>
+        <v>179</v>
       </c>
       <c r="AB39" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="40" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="AC39" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="12" t="str">
+        <f>VLOOKUP(A40,Sheet2!B40:B82,1,0)</f>
+        <v>ASA102</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C40">
-        <v>0</v>
-      </c>
       <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
         <v>45995.4</v>
-      </c>
-      <c r="G40">
-        <v>11498.85</v>
       </c>
       <c r="H40">
         <v>11498.85</v>
@@ -3406,109 +3598,117 @@
       <c r="J40">
         <v>11498.85</v>
       </c>
-      <c r="K40" t="s">
+      <c r="K40">
+        <v>11498.85</v>
+      </c>
+      <c r="L40" t="s">
         <v>27</v>
       </c>
-      <c r="N40" s="3">
+      <c r="O40" s="3">
         <v>43971</v>
       </c>
-      <c r="R40" t="s">
-        <v>99</v>
-      </c>
-      <c r="V40" t="s">
-        <v>103</v>
+      <c r="S40" t="s">
+        <v>98</v>
       </c>
       <c r="W40" t="s">
+        <v>102</v>
+      </c>
+      <c r="X40" t="s">
         <v>71</v>
       </c>
-      <c r="X40" t="s">
-        <v>140</v>
-      </c>
       <c r="Y40" t="s">
+        <v>139</v>
+      </c>
+      <c r="Z40" t="s">
         <v>28</v>
       </c>
-      <c r="Z40" t="s">
-        <v>181</v>
-      </c>
       <c r="AA40" t="s">
-        <v>228</v>
-      </c>
-      <c r="AB40">
+        <v>180</v>
+      </c>
+      <c r="AB40" t="s">
+        <v>225</v>
+      </c>
+      <c r="AC40">
         <v>104935171</v>
       </c>
     </row>
-    <row r="41" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="12" t="e">
+        <f>VLOOKUP(A41,Sheet2!B41:B83,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
       <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
         <v>38915.949999999997</v>
-      </c>
-      <c r="G41">
-        <v>6896.55</v>
       </c>
       <c r="H41">
         <v>6896.55</v>
       </c>
       <c r="I41">
+        <v>6896.55</v>
+      </c>
+      <c r="J41">
         <v>4597.7</v>
       </c>
-      <c r="J41">
+      <c r="K41">
         <v>20525.150000000001</v>
       </c>
-      <c r="K41" t="s">
+      <c r="L41" t="s">
         <v>27</v>
       </c>
-      <c r="N41" s="3">
+      <c r="O41" s="3">
         <v>46527</v>
       </c>
-      <c r="R41" t="s">
-        <v>95</v>
-      </c>
-      <c r="V41" t="s">
-        <v>103</v>
+      <c r="S41" t="s">
+        <v>94</v>
       </c>
       <c r="W41" t="s">
+        <v>102</v>
+      </c>
+      <c r="X41" t="s">
         <v>72</v>
       </c>
-      <c r="X41" t="s">
-        <v>139</v>
-      </c>
       <c r="Y41" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z41" t="s">
         <v>28</v>
       </c>
-      <c r="Z41" t="s">
-        <v>89</v>
-      </c>
       <c r="AA41" t="s">
-        <v>229</v>
-      </c>
-      <c r="AB41">
+        <v>88</v>
+      </c>
+      <c r="AB41" t="s">
+        <v>226</v>
+      </c>
+      <c r="AC41">
         <v>115758281</v>
       </c>
     </row>
-    <row r="42" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="12" t="e">
+        <f>VLOOKUP(A42,Sheet2!B42:B84,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
       <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
         <v>36460.5</v>
       </c>
-      <c r="G42">
-        <v>0</v>
-      </c>
       <c r="H42">
         <v>0</v>
       </c>
@@ -3516,322 +3716,346 @@
         <v>0</v>
       </c>
       <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
         <v>36460.5</v>
       </c>
-      <c r="K42" t="s">
+      <c r="L42" t="s">
         <v>27</v>
       </c>
-      <c r="R42" t="s">
-        <v>99</v>
-      </c>
-      <c r="V42" t="s">
-        <v>103</v>
+      <c r="S42" t="s">
+        <v>98</v>
       </c>
       <c r="W42" t="s">
+        <v>102</v>
+      </c>
+      <c r="X42" t="s">
         <v>73</v>
       </c>
-      <c r="X42" t="s">
-        <v>141</v>
-      </c>
       <c r="Y42" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z42" t="s">
         <v>28</v>
       </c>
-      <c r="Z42" t="s">
-        <v>182</v>
-      </c>
       <c r="AA42" t="s">
-        <v>230</v>
-      </c>
-      <c r="AB42">
+        <v>181</v>
+      </c>
+      <c r="AB42" t="s">
+        <v>227</v>
+      </c>
+      <c r="AC42">
         <v>216716791</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="12" t="e">
+        <f>VLOOKUP(A43,Sheet2!B43:B85,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
       <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
         <v>771839.75</v>
       </c>
-      <c r="G43">
+      <c r="H43">
         <v>75981.19</v>
       </c>
-      <c r="H43">
+      <c r="I43">
         <v>68308.55</v>
       </c>
-      <c r="I43">
+      <c r="J43">
         <v>69242.27</v>
       </c>
-      <c r="J43">
+      <c r="K43">
         <v>558307.74</v>
       </c>
-      <c r="K43" t="s">
+      <c r="L43" t="s">
         <v>27</v>
       </c>
-      <c r="R43" t="s">
-        <v>95</v>
-      </c>
-      <c r="V43" t="s">
-        <v>103</v>
+      <c r="S43" t="s">
+        <v>94</v>
       </c>
       <c r="W43" t="s">
+        <v>102</v>
+      </c>
+      <c r="X43" t="s">
         <v>74</v>
       </c>
-      <c r="X43" t="s">
-        <v>142</v>
-      </c>
       <c r="Y43" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="Z43" t="s">
-        <v>87</v>
+        <v>168</v>
       </c>
       <c r="AA43" t="s">
-        <v>231</v>
-      </c>
-      <c r="AB43">
+        <v>86</v>
+      </c>
+      <c r="AB43" t="s">
+        <v>228</v>
+      </c>
+      <c r="AC43">
         <v>113211761</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="12" t="e">
+        <f>VLOOKUP(A44,Sheet2!B44:B86,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
       <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
         <v>329214.55</v>
       </c>
-      <c r="G44">
+      <c r="H44">
         <v>266053.38</v>
       </c>
-      <c r="H44">
-        <v>0</v>
-      </c>
       <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
         <v>63161.17</v>
       </c>
-      <c r="J44">
-        <v>0</v>
-      </c>
-      <c r="K44" t="s">
+      <c r="K44">
+        <v>0</v>
+      </c>
+      <c r="L44" t="s">
         <v>27</v>
       </c>
-      <c r="N44" s="3">
+      <c r="O44" s="3">
         <v>43636</v>
       </c>
-      <c r="R44" t="s">
-        <v>95</v>
-      </c>
-      <c r="V44" t="s">
-        <v>103</v>
+      <c r="S44" t="s">
+        <v>94</v>
       </c>
       <c r="W44" t="s">
+        <v>102</v>
+      </c>
+      <c r="X44" t="s">
         <v>75</v>
       </c>
-      <c r="X44" t="s">
-        <v>143</v>
-      </c>
       <c r="Y44" t="s">
+        <v>142</v>
+      </c>
+      <c r="Z44" t="s">
         <v>28</v>
       </c>
-      <c r="Z44" t="s">
-        <v>183</v>
-      </c>
       <c r="AA44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB44">
+        <v>182</v>
+      </c>
+      <c r="AB44" t="s">
+        <v>229</v>
+      </c>
+      <c r="AC44">
         <v>123198870</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="12" t="e">
+        <f>VLOOKUP(A45,Sheet2!B45:B87,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C45">
-        <v>0</v>
-      </c>
       <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
         <v>219575.53</v>
       </c>
-      <c r="G45">
+      <c r="H45">
         <v>14431.78</v>
       </c>
-      <c r="H45">
+      <c r="I45">
         <v>19101.189999999999</v>
       </c>
-      <c r="I45">
+      <c r="J45">
         <v>19650.89</v>
       </c>
-      <c r="J45">
+      <c r="K45">
         <v>166391.67000000001</v>
       </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
         <v>27</v>
       </c>
-      <c r="N45" s="3">
+      <c r="O45" s="3">
         <v>45402</v>
       </c>
-      <c r="R45" t="s">
-        <v>95</v>
-      </c>
-      <c r="V45" t="s">
-        <v>103</v>
+      <c r="S45" t="s">
+        <v>94</v>
       </c>
       <c r="W45" t="s">
+        <v>102</v>
+      </c>
+      <c r="X45" t="s">
         <v>76</v>
       </c>
-      <c r="X45" t="s">
-        <v>144</v>
-      </c>
       <c r="Y45" t="s">
+        <v>143</v>
+      </c>
+      <c r="Z45" t="s">
         <v>28</v>
       </c>
-      <c r="Z45" t="s">
-        <v>184</v>
-      </c>
       <c r="AA45" t="s">
-        <v>233</v>
+        <v>183</v>
       </c>
       <c r="AB45" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="46" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+      <c r="AC45" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="46" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="12" t="e">
+        <f>VLOOKUP(A46,Sheet2!B46:B88,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C46">
-        <v>0</v>
-      </c>
       <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
         <v>133805.12</v>
       </c>
-      <c r="G46">
+      <c r="H46">
         <v>68890.039999999994</v>
       </c>
-      <c r="H46">
+      <c r="I46">
         <v>39402.03</v>
       </c>
-      <c r="I46">
+      <c r="J46">
         <v>9266.44</v>
       </c>
-      <c r="J46">
+      <c r="K46">
         <v>16246.61</v>
       </c>
-      <c r="K46" t="s">
+      <c r="L46" t="s">
         <v>27</v>
       </c>
-      <c r="R46" t="s">
-        <v>100</v>
-      </c>
-      <c r="V46" t="s">
-        <v>103</v>
+      <c r="S46" t="s">
+        <v>99</v>
       </c>
       <c r="W46" t="s">
+        <v>102</v>
+      </c>
+      <c r="X46" t="s">
         <v>77</v>
       </c>
-      <c r="X46" t="s">
-        <v>145</v>
-      </c>
       <c r="Y46" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z46" t="s">
         <v>28</v>
       </c>
-      <c r="Z46" t="s">
-        <v>185</v>
-      </c>
       <c r="AA46" t="s">
-        <v>234</v>
-      </c>
-      <c r="AB46">
+        <v>184</v>
+      </c>
+      <c r="AB46" t="s">
+        <v>231</v>
+      </c>
+      <c r="AC46">
         <v>126647823</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="12" t="e">
+        <f>VLOOKUP(A47,Sheet2!B47:B89,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C47">
-        <v>0</v>
-      </c>
       <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
         <v>52875.85</v>
       </c>
-      <c r="G47">
+      <c r="H47">
         <v>17241.95</v>
-      </c>
-      <c r="H47">
-        <v>17816.95</v>
       </c>
       <c r="I47">
         <v>17816.95</v>
       </c>
       <c r="J47">
-        <v>0</v>
-      </c>
-      <c r="K47" t="s">
+        <v>17816.95</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+      <c r="L47" t="s">
         <v>27</v>
       </c>
-      <c r="R47" t="s">
-        <v>87</v>
-      </c>
-      <c r="V47" t="s">
-        <v>103</v>
+      <c r="S47" t="s">
+        <v>86</v>
       </c>
       <c r="W47" t="s">
+        <v>102</v>
+      </c>
+      <c r="X47" t="s">
         <v>78</v>
       </c>
-      <c r="X47" t="s">
-        <v>139</v>
-      </c>
       <c r="Y47" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z47" t="s">
         <v>28</v>
       </c>
-      <c r="Z47" t="s">
-        <v>180</v>
-      </c>
       <c r="AA47" t="s">
-        <v>235</v>
-      </c>
-      <c r="AB47">
+        <v>179</v>
+      </c>
+      <c r="AB47" t="s">
+        <v>232</v>
+      </c>
+      <c r="AC47">
         <v>115757749</v>
       </c>
     </row>
-    <row r="48" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="12" t="e">
+        <f>VLOOKUP(A48,Sheet2!B48:B90,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C48">
-        <v>0</v>
-      </c>
       <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
         <v>48300</v>
-      </c>
-      <c r="G48">
-        <v>16100</v>
       </c>
       <c r="H48">
         <v>16100</v>
@@ -3840,199 +4064,755 @@
         <v>16100</v>
       </c>
       <c r="J48">
-        <v>0</v>
-      </c>
-      <c r="K48" t="s">
+        <v>16100</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
+      <c r="L48" t="s">
         <v>27</v>
       </c>
-      <c r="R48" t="s">
-        <v>101</v>
-      </c>
-      <c r="V48" t="s">
-        <v>103</v>
+      <c r="S48" t="s">
+        <v>100</v>
       </c>
       <c r="W48" t="s">
+        <v>102</v>
+      </c>
+      <c r="X48" t="s">
         <v>79</v>
       </c>
-      <c r="X48" t="s">
-        <v>146</v>
-      </c>
       <c r="Y48" t="s">
+        <v>145</v>
+      </c>
+      <c r="Z48" t="s">
         <v>28</v>
       </c>
-      <c r="Z48" t="s">
-        <v>186</v>
-      </c>
       <c r="AA48" t="s">
-        <v>236</v>
-      </c>
-      <c r="AB48">
+        <v>185</v>
+      </c>
+      <c r="AB48" t="s">
+        <v>233</v>
+      </c>
+      <c r="AC48">
         <v>644975798</v>
       </c>
     </row>
-    <row r="49" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B49" s="10" t="s">
+      <c r="B49" s="12" t="e">
+        <f>VLOOKUP(A49,Sheet2!B49:B91,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C49">
-        <v>0</v>
-      </c>
       <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
         <v>42611.72</v>
       </c>
-      <c r="G49">
+      <c r="H49">
         <v>21652.97</v>
       </c>
-      <c r="H49">
+      <c r="I49">
         <v>20958.75</v>
       </c>
-      <c r="I49">
-        <v>0</v>
-      </c>
       <c r="J49">
         <v>0</v>
       </c>
-      <c r="K49" t="s">
+      <c r="K49">
+        <v>0</v>
+      </c>
+      <c r="L49" t="s">
         <v>27</v>
       </c>
-      <c r="N49" s="3">
+      <c r="O49" s="3">
         <v>11129</v>
       </c>
-      <c r="R49" t="s">
-        <v>95</v>
-      </c>
-      <c r="V49" t="s">
-        <v>103</v>
+      <c r="S49" t="s">
+        <v>94</v>
       </c>
       <c r="W49" t="s">
+        <v>102</v>
+      </c>
+      <c r="X49" t="s">
         <v>80</v>
       </c>
-      <c r="X49" t="s">
-        <v>147</v>
-      </c>
       <c r="Y49" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z49" t="s">
         <v>28</v>
       </c>
-      <c r="Z49" t="s">
-        <v>187</v>
-      </c>
       <c r="AA49" t="s">
-        <v>237</v>
-      </c>
-      <c r="AB49">
+        <v>186</v>
+      </c>
+      <c r="AB49" t="s">
+        <v>234</v>
+      </c>
+      <c r="AC49">
         <v>115462117</v>
       </c>
     </row>
-    <row r="50" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="10" t="s">
+      <c r="B50" s="12" t="e">
+        <f>VLOOKUP(A50,Sheet2!B50:B92,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
       <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
         <v>38425.75</v>
       </c>
-      <c r="G50">
+      <c r="H50">
         <v>38425.75</v>
       </c>
-      <c r="H50">
-        <v>0</v>
-      </c>
       <c r="I50">
         <v>0</v>
       </c>
       <c r="J50">
         <v>0</v>
       </c>
-      <c r="K50" t="s">
+      <c r="K50">
+        <v>0</v>
+      </c>
+      <c r="L50" t="s">
         <v>27</v>
       </c>
-      <c r="R50" t="s">
-        <v>95</v>
-      </c>
-      <c r="V50" t="s">
-        <v>103</v>
+      <c r="S50" t="s">
+        <v>94</v>
       </c>
       <c r="W50" t="s">
+        <v>102</v>
+      </c>
+      <c r="X50" t="s">
         <v>81</v>
       </c>
-      <c r="X50" t="s">
-        <v>148</v>
-      </c>
       <c r="Y50" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="Z50" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="AA50" t="s">
-        <v>238</v>
-      </c>
-      <c r="AB50">
+        <v>86</v>
+      </c>
+      <c r="AB50" t="s">
+        <v>235</v>
+      </c>
+      <c r="AC50">
         <v>105932665</v>
       </c>
     </row>
-    <row r="51" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="12" t="e">
+        <f>VLOOKUP(A51,Sheet2!B51:B93,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C51" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
       <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
         <v>35696.86</v>
       </c>
-      <c r="G51">
+      <c r="H51">
         <v>1127</v>
       </c>
-      <c r="H51">
+      <c r="I51">
         <v>2254</v>
       </c>
-      <c r="I51">
-        <v>0</v>
-      </c>
       <c r="J51">
+        <v>0</v>
+      </c>
+      <c r="K51">
         <v>32315.86</v>
       </c>
-      <c r="K51" t="s">
+      <c r="L51" t="s">
         <v>27</v>
       </c>
-      <c r="R51" t="s">
-        <v>102</v>
-      </c>
-      <c r="V51" t="s">
-        <v>103</v>
+      <c r="S51" t="s">
+        <v>101</v>
       </c>
       <c r="W51" t="s">
+        <v>102</v>
+      </c>
+      <c r="X51" t="s">
         <v>82</v>
       </c>
-      <c r="X51" t="s">
+      <c r="Y51" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z51" t="s">
         <v>149</v>
       </c>
-      <c r="Y51" t="s">
-        <v>150</v>
-      </c>
-      <c r="Z51" t="s">
-        <v>188</v>
-      </c>
       <c r="AA51" t="s">
-        <v>239</v>
-      </c>
-      <c r="AB51">
+        <v>187</v>
+      </c>
+      <c r="AB51" t="s">
+        <v>236</v>
+      </c>
+      <c r="AC51">
         <v>871350000</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC51" xr:uid="{0C3DA5CB-527D-B84B-8680-044C20C86614}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="#N/A"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48D823A6-8EDE-6547-9B16-E330DA46123A}">
+  <dimension ref="A1:C44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="41" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="str">
+        <f>VLOOKUP(Sheet2!B2,Sheet1!A2:A51,1,0)</f>
+        <v>ZOOM01</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="str">
+        <f>VLOOKUP(Sheet2!B3,Sheet1!A3:A52,1,0)</f>
+        <v>XPE101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="str">
+        <f>VLOOKUP(Sheet2!B4,Sheet1!A4:A53,1,0)</f>
+        <v>WEB101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="str">
+        <f>VLOOKUP(Sheet2!B5,Sheet1!A5:A54,1,0)</f>
+        <v>VOX101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="str">
+        <f>VLOOKUP(Sheet2!B6,Sheet1!A6:A55,1,0)</f>
+        <v>VOD101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" t="str">
+        <f>VLOOKUP(Sheet2!B7,Sheet1!A7:A56,1,0)</f>
+        <v>ITHE01</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="str">
+        <f>VLOOKUP(Sheet2!B8,Sheet1!A8:A57,1,0)</f>
+        <v>BSIT01</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="str">
+        <f>VLOOKUP(Sheet2!B9,Sheet1!A9:A58,1,0)</f>
+        <v>SUPE01</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" t="str">
+        <f>VLOOKUP(Sheet2!B10,Sheet1!A10:A59,1,0)</f>
+        <v>GLG101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="e">
+        <f>VLOOKUP(Sheet2!B11,Sheet1!A11:A60,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" t="str">
+        <f>VLOOKUP(Sheet2!B12,Sheet1!A12:A61,1,0)</f>
+        <v>SERA02</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" t="str">
+        <f>VLOOKUP(Sheet2!B13,Sheet1!A13:A62,1,0)</f>
+        <v>CITY01</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="e">
+        <f>VLOOKUP(Sheet2!B14,Sheet1!A14:A63,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" t="str">
+        <f>VLOOKUP(Sheet2!B15,Sheet1!A15:A64,1,0)</f>
+        <v>REAL01</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C16" t="e">
+        <f>VLOOKUP(Sheet2!B16,Sheet1!A16:A65,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="e">
+        <f>VLOOKUP(Sheet2!B17,Sheet1!A17:A66,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" t="str">
+        <f>VLOOKUP(Sheet2!B18,Sheet1!A18:A67,1,0)</f>
+        <v>MTN102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" t="str">
+        <f>VLOOKUP(Sheet2!B19,Sheet1!A19:A68,1,0)</f>
+        <v>MGC101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" t="str">
+        <f>VLOOKUP(Sheet2!B20,Sheet1!A20:A69,1,0)</f>
+        <v>MAN107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="str">
+        <f>VLOOKUP(Sheet2!B21,Sheet1!A21:A70,1,0)</f>
+        <v>LIQ103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" t="e">
+        <f>VLOOKUP(Sheet2!B22,Sheet1!A22:A71,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" t="e">
+        <f>VLOOKUP(Sheet2!B23,Sheet1!A23:A72,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" t="e">
+        <f>VLOOKUP(Sheet2!B24,Sheet1!A24:A73,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" t="str">
+        <f>VLOOKUP(Sheet2!B25,Sheet1!A25:A74,1,0)</f>
+        <v>INT104</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" t="str">
+        <f>VLOOKUP(Sheet2!B26,Sheet1!A26:A75,1,0)</f>
+        <v>INT107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>138</v>
+      </c>
+      <c r="B27" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" t="str">
+        <f>VLOOKUP(Sheet2!B27,Sheet1!A27:A76,1,0)</f>
+        <v>INTKC1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="e">
+        <f>VLOOKUP(Sheet2!B28,Sheet1!A28:A77,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" t="str">
+        <f>VLOOKUP(Sheet2!B29,Sheet1!A29:A78,1,0)</f>
+        <v>HIT101</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>128</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" t="e">
+        <f>VLOOKUP(Sheet2!B30,Sheet1!A30:A79,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" t="e">
+        <f>VLOOKUP(Sheet2!B31,Sheet1!A31:A80,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="e">
+        <f>VLOOKUP(Sheet2!B32,Sheet1!A32:A81,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>105</v>
+      </c>
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" t="e">
+        <f>VLOOKUP(Sheet2!B33,Sheet1!A33:A82,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" t="e">
+        <f>VLOOKUP(Sheet2!B34,Sheet1!A34:A83,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>147</v>
+      </c>
+      <c r="B35" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" t="str">
+        <f>VLOOKUP(Sheet2!B35,Sheet1!A35:A84,1,0)</f>
+        <v>COO101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C36" t="e">
+        <f>VLOOKUP(Sheet2!B36,Sheet1!A36:A85,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>148</v>
+      </c>
+      <c r="B37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" t="str">
+        <f>VLOOKUP(Sheet2!B37,Sheet1!A37:A86,1,0)</f>
+        <v>BITC01</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>140</v>
+      </c>
+      <c r="B38" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" t="str">
+        <f>VLOOKUP(Sheet2!B38,Sheet1!A38:A87,1,0)</f>
+        <v>BGR101</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>110</v>
+      </c>
+      <c r="B39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" t="e">
+        <f>VLOOKUP(Sheet2!B39,Sheet1!A39:A88,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" t="e">
+        <f>VLOOKUP(Sheet2!B40,Sheet1!A40:A89,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" t="e">
+        <f>VLOOKUP(Sheet2!B41,Sheet1!A41:A90,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" t="e">
+        <f>VLOOKUP(Sheet2!B42,Sheet1!A42:A91,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>139</v>
+      </c>
+      <c r="B43" t="s">
+        <v>71</v>
+      </c>
+      <c r="C43" t="e">
+        <f>VLOOKUP(Sheet2!B43,Sheet1!A43:A92,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" t="s">
+        <v>51</v>
+      </c>
+      <c r="C44" t="e">
+        <f>VLOOKUP(Sheet2!B44,Sheet1!A44:A93,1,0)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C44" xr:uid="{DB86DBB2-B4C7-4245-AD01-D14C1594D246}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finally gone live - drawing a line in the sand for everything that works
</commit_message>
<xml_diff>
--- a/documents/SADV collections upload.xlsx
+++ b/documents/SADV collections upload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC881B-6BCF-AA4C-88B6-58FDB91C6689}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534F471E-234E-E143-B2F2-3115B737175D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="960" windowWidth="27640" windowHeight="16000" xr2:uid="{B1A7F133-870B-BE4E-A664-D1E75F837A44}"/>
   </bookViews>
@@ -1412,7 +1412,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1556,7 +1556,7 @@
         <v>114695876</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>786737791</v>
       </c>
     </row>
-    <row r="8" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>119797038</v>
       </c>
     </row>
-    <row r="13" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>44</v>
       </c>
@@ -2018,7 +2018,7 @@
         <v>214649682</v>
       </c>
     </row>
-    <row r="14" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>45</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>848373798</v>
       </c>
     </row>
-    <row r="15" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>46</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>214649682</v>
       </c>
     </row>
-    <row r="16" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>47</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>100150150</v>
       </c>
     </row>
-    <row r="23" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>54</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>791494245</v>
       </c>
     </row>
-    <row r="25" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>56</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="26" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>57</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>124431000</v>
       </c>
     </row>
-    <row r="27" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>58</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>828517094</v>
       </c>
     </row>
-    <row r="29" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>60</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>115193000</v>
       </c>
     </row>
-    <row r="30" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>61</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>115851000</v>
       </c>
     </row>
-    <row r="31" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>62</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>604821967</v>
       </c>
     </row>
-    <row r="32" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>63</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>114474360</v>
       </c>
     </row>
-    <row r="33" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>64</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="35" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
@@ -3338,7 +3338,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="36" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>67</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>117450100</v>
       </c>
     </row>
-    <row r="37" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>68</v>
       </c>
@@ -3455,7 +3455,7 @@
         <v>119123000</v>
       </c>
     </row>
-    <row r="38" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>69</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>100107301</v>
       </c>
     </row>
-    <row r="39" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>70</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>104935171</v>
       </c>
     </row>
-    <row r="41" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>72</v>
       </c>
@@ -3692,7 +3692,7 @@
         <v>115758281</v>
       </c>
     </row>
-    <row r="42" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>73</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>216716791</v>
       </c>
     </row>
-    <row r="43" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>74</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>113211761</v>
       </c>
     </row>
-    <row r="44" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>75</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>123198870</v>
       </c>
     </row>
-    <row r="45" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>76</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="46" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>77</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>126647823</v>
       </c>
     </row>
-    <row r="47" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>78</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>115757749</v>
       </c>
     </row>
-    <row r="48" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>79</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>644975798</v>
       </c>
     </row>
-    <row r="49" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>80</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>115462117</v>
       </c>
     </row>
-    <row r="50" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>81</v>
       </c>
@@ -4214,7 +4214,7 @@
         <v>105932665</v>
       </c>
     </row>
-    <row r="51" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:29" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>82</v>
       </c>
@@ -4273,9 +4273,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AC51" xr:uid="{0C3DA5CB-527D-B84B-8680-044C20C86614}">
-    <filterColumn colId="1">
+    <filterColumn colId="24">
       <filters>
-        <filter val="#N/A"/>
+        <filter val="SERENGETI GOLF &amp; WILDLIFE EST. MARKETING"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>